<commit_message>
feat(data): research source catalogue facts
</commit_message>
<xml_diff>
--- a/data/variables_catalogue.xlsx
+++ b/data/variables_catalogue.xlsx
@@ -643,9 +643,6 @@
           <t>Total administrative area of the Kreis</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -688,9 +685,6 @@
           <t>Total area used for agriculture</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -733,9 +727,6 @@
           <t>Agricultural area as % of total area (derived)</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -778,9 +769,6 @@
           <t>Arable / cropland area</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -823,9 +811,6 @@
           <t>Permanent pastures and meadows</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -868,9 +853,6 @@
           <t>Area planted with vines</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -913,9 +895,6 @@
           <t>Fruit trees, nurseries and other permanent crops</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -958,9 +937,6 @@
           <t>Total number of agricultural holdings</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1003,9 +979,6 @@
           <t>Total UAA across all farms</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1048,9 +1021,6 @@
           <t>UAA / farms count (derived)</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1093,9 +1063,6 @@
           <t>Number of certified organic farms</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1138,9 +1105,6 @@
           <t>UAA under organic management</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1183,9 +1147,6 @@
           <t>Organic UAA as % of total UAA (derived)</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1228,9 +1189,6 @@
           <t>UAA farmed by the owner</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1273,9 +1231,6 @@
           <t>UAA under tenancy/lease</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1318,9 +1273,6 @@
           <t>Rented UAA as % of total UAA (derived)</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1363,9 +1315,6 @@
           <t>Holdings with UAA below 5 ha</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1408,9 +1357,6 @@
           <t>Holdings with UAA 5 to 20 ha</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1453,9 +1399,6 @@
           <t>Holdings with UAA 20 to 50 ha</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1498,9 +1441,6 @@
           <t>Holdings with UAA 50 to 100 ha</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1543,9 +1483,6 @@
           <t>Holdings with UAA above 100 ha</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1588,9 +1525,6 @@
           <t>Full-time equivalent farm labour</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1633,9 +1567,6 @@
           <t>Area sown with cereals (wheat, rye, barley, etc.)</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1678,9 +1609,6 @@
           <t>Rapeseed, sunflower and other oilseeds</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1723,9 +1651,6 @@
           <t>Area under sugar beet</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1768,9 +1693,6 @@
           <t>Open-field and glasshouse vegetables</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1813,9 +1735,6 @@
           <t>Total maize area</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1858,9 +1777,6 @@
           <t>All species expressed in livestock units</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1903,9 +1819,6 @@
           <t>LU per ha UAA (derived)</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1948,9 +1861,6 @@
           <t>Total cattle including dairy cows</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1993,9 +1903,6 @@
           <t>Cows kept for milk production</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2038,9 +1945,6 @@
           <t>Total swine headcount</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2083,9 +1987,6 @@
           <t>All poultry species</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2128,9 +2029,6 @@
           <t>N input minus N output per ha UAA</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2173,9 +2071,6 @@
           <t>P input minus P output per ha UAA</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2218,9 +2113,6 @@
           <t>Total pesticide active ingredients sold in Kreis</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2263,9 +2155,6 @@
           <t>Area receiving supplementary irrigation</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2308,9 +2197,6 @@
           <t>Total volume of water applied for irrigation</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2353,9 +2239,6 @@
           <t>Average price per ha of sold agricultural land</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2398,9 +2281,6 @@
           <t>Average annual rent per ha of leased agricultural land</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2443,9 +2323,6 @@
           <t>Total forest and woodland area</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2488,9 +2365,6 @@
           <t>Forest owned by state/municipality as % of total forest</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2533,9 +2407,6 @@
           <t>Area designated under EU Habitats or Birds Directive</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2578,9 +2449,6 @@
           <t>Strictly protected nature reserve area</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2623,9 +2491,6 @@
           <t>Less-strict landscape protection zones</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2668,9 +2533,6 @@
           <t>Methane from livestock and manure management</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2713,9 +2575,6 @@
           <t>Nitrous oxide from soils and fertiliser application</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2758,9 +2617,6 @@
           <t>Average nitrate concentration at monitoring stations</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2803,9 +2659,6 @@
           <t>Built-up land including roads and railways</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2848,9 +2701,6 @@
           <t>Sealed/impervious surface as % of total area</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2893,9 +2743,6 @@
           <t>Resident population at year-end</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2938,9 +2785,6 @@
           <t>Population per km2 (derived)</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2983,9 +2827,6 @@
           <t>Number of live births per year</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3028,9 +2869,6 @@
           <t>Number of deaths per year</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3073,9 +2911,6 @@
           <t>Births minus deaths</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3118,9 +2953,6 @@
           <t>In-migrants minus out-migrants</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3163,9 +2995,6 @@
           <t>Children and youth as % of total population</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3208,9 +3037,6 @@
           <t>Elderly population share - indicator of rural ageing</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3253,9 +3079,6 @@
           <t>Population aged 18-64 as % of total</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3298,9 +3121,6 @@
           <t>Non-German residents as % of total population</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3343,9 +3163,6 @@
           <t>Gross domestic product per resident</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3388,9 +3205,6 @@
           <t>Agriculture, forestry and fishing share of total GVA</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3433,9 +3247,6 @@
           <t>Manufacturing and mining share of total GVA</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3478,9 +3289,6 @@
           <t>Services share of total GVA</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3523,9 +3331,6 @@
           <t>Net income available to households per resident</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3568,9 +3373,6 @@
           <t>Unemployed as % of civilian labour force</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3613,9 +3415,6 @@
           <t>Unemployed aged 15-25 as % of that age group</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3658,9 +3457,6 @@
           <t>Workers commuting into the Kreis</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3703,9 +3499,6 @@
           <t>Workers commuting out of the Kreis</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3748,9 +3541,6 @@
           <t>In-commuters minus out-commuters (derived)</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3766,7 +3556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3879,7 +3669,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>agraratlas_wcs</t>
+          <t>agraratlas_wcs_farm_structure</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3894,7 +3684,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LL-relevant WCS coverages</t>
+          <t>Farm-structure WCS coverages</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3902,8 +3692,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2010, 2016, 2020 census years</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>WCS</t>
@@ -3914,18 +3712,46 @@
           <t>https://www.wcs.nrw.de/stba/agraratlas?REQUEST=getCapabilities&amp;SERVICE=WCS&amp;VERSION=1.0.0</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>WCS raster coverages</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>https://www.wcs.nrw.de/stba/agraratlas?REQUEST=getCapabilities&amp;SERVICE=WCS&amp;VERSION=1.0.0</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>All 5 LLs; tabular/raster statistics can be filtered to LL NUTS-3 regions after download</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>tabular</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Large WCS bounded to farm-structure themes; kind: tabular does not yet exist in sources.yaml.</t>
+        </is>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
@@ -3934,7 +3760,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>destatis_genesis</t>
+          <t>agraratlas_wcs_organic</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3944,62 +3770,62 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DESTATIS GENESIS</t>
+          <t>Agraratlas Statistikportal</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NUTS-3 statistical variables</t>
+          <t>Organic farming WCS coverages</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>in-progress</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Germany, administrative statistics</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>varies by GENESIS table</t>
+          <t>2010, 2016, 2020 census years</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>REST-item</t>
+          <t>WCS</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www-genesis.destatis.de/datenbank/online</t>
+          <t>https://www.wcs.nrw.de/stba/agraratlas?REQUEST=getCapabilities&amp;SERVICE=WCS&amp;VERSION=1.0.0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>JSON/CSV via GENESIS API</t>
+          <t>WCS raster coverages</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>API terms; token required</t>
+          <t>[needs-verification]</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>varies by table</t>
+          <t>[needs-verification]</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>https://www-genesis.destatis.de/datenbank/online</t>
+          <t>https://www.wcs.nrw.de/stba/agraratlas?REQUEST=getCapabilities&amp;SERVICE=WCS&amp;VERSION=1.0.0</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>All 5 LLs via NUTS-3 statistics</t>
+          <t>All 5 LLs; useful for organic-farming comparison across LL regions</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -4014,14 +3840,10 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Pipeline is in progress; auth token must never be committed.</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>include</t>
-        </is>
-      </c>
+          <t>Large WCS bounded to organic-farming themes; kind: tabular does not yet exist in sources.yaml.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -4029,54 +3851,94 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>degree_urbanisation</t>
+          <t>destatis_genesis</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Demographics / Settlement</t>
+          <t>Agricultural Statistics</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GHSL Degree of Urbanisation</t>
+          <t>DESTATIS GENESIS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Degree of Urbanisation classification</t>
+          <t>NUTS-3 statistical variables</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+          <t>in-progress</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Germany, administrative statistics</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>varies by GENESIS table</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>manual-download</t>
+          <t>REST-item</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://ghsl.jrc.ec.europa.eu/download.php</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
+          <t>https://www-genesis.destatis.de/datenbank/online</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>JSON/CSV via GENESIS API</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>API terms; token required</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>varies by table</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>https://ghsl.jrc.ec.europa.eu/download.php</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
+          <t>https://www-genesis.destatis.de/datenbank/online</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>All 5 LLs via NUTS-3 statistics</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>tabular</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Pipeline is in progress; auth token must never be committed.</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -4084,22 +3946,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>dwd_cdc_daily_precipitation</t>
+          <t>degree_urbanisation</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Climate</t>
+          <t>Demographics / Settlement</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DWD Climate Data Center</t>
+          <t>GHSL Degree of Urbanisation</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Daily precipitation station data</t>
+          <t>Degree of Urbanisation classification</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -4107,30 +3969,66 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Global; country and tile downloads available</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>multiple epochs/resolutions depending on product</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>FTP</t>
+          <t>manual-download</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://opendata.dwd.de/climate_environment/CDC/</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
+          <t>https://ghsl.jrc.ec.europa.eu/download.php</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>ZIP downloads with vector boundaries and classification tables</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>European Union reuse with proper acknowledgement</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>updated releases; product-specific</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>https://opendata.dwd.de/climate_environment/CDC/Readme_intro_CDC_ftp.txt</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
+          <t>https://ghsl.jrc.ec.europa.eu/download.php</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>All 5 LLs; settlement context around rural/agricultural LL regions</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>tabular</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Manual GHSL product selection; likely use country split/table join rather than full global rasters.</t>
+        </is>
+      </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
@@ -4139,7 +4037,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>dwd_cdc_daily_temperature</t>
+          <t>dwd_cdc_daily_precipitation</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4154,7 +4052,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Daily temperature station data</t>
+          <t>Daily precipitation station data</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4162,8 +4060,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>historical and recent station time series</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>FTP</t>
@@ -4174,18 +4080,46 @@
           <t>https://opendata.dwd.de/climate_environment/CDC/</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ZIP archives with station metadata/text tables</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>open data; cite DWD terms</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>ongoing CDC updates</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr">
         <is>
           <t>https://opendata.dwd.de/climate_environment/CDC/Readme_intro_CDC_ftp.txt</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>All 5 LLs via station filtering or interpolation to LL regions</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>tabular</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Bounded CDC entry; do not enumerate all DWD parameters.</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
@@ -4194,7 +4128,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dwd_cdc_gridded_precipitation</t>
+          <t>dwd_cdc_daily_temperature</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4209,7 +4143,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>HYRAS gridded precipitation</t>
+          <t>Daily temperature station data</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4217,8 +4151,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>historical and recent station time series</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>FTP</t>
@@ -4229,18 +4171,46 @@
           <t>https://opendata.dwd.de/climate_environment/CDC/</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>ZIP archives with station metadata/text tables</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>open data; cite DWD terms</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>ongoing CDC updates</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>https://opendata.dwd.de/climate_environment/CDC/Readme_intro_CDC_ftp.txt</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>All 5 LLs via station filtering or interpolation to LL regions</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>tabular</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Bounded CDC entry; do not enumerate all DWD parameters.</t>
+        </is>
+      </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
@@ -4249,27 +4219,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>buek250_soil</t>
+          <t>dwd_cdc_gridded_precipitation</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Existing Integrations</t>
+          <t>Climate</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BUEK250 Soil</t>
+          <t>DWD Climate Data Center</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BUEK250 soil polygons</t>
+          <t>HYRAS gridded precipitation</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -4279,64 +4249,60 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>static federal soil map</t>
+          <t>historical gridded precipitation product</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>manual-download</t>
+          <t>FTP</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://www.bgr.bund.de/DE/Themen/Boden/Informationsgrundlagen/Bodenkundliche_Karten_Datenbanken/BUEK250/buek250_node.html</t>
+          <t>https://opendata.dwd.de/climate_environment/CDC/</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>GeoPackage/GeoJSON</t>
+          <t>gridded raster archives</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>GeoNutzV/DL-DE-BY style terms</t>
+          <t>open data; cite DWD terms</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>static</t>
+          <t>product-specific updates</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://www.bgr.bund.de/DE/Themen/Boden/Informationsgrundlagen/Bodenkundliche_Karten_Datenbanken/BUEK250/buek250_node.html</t>
+          <t>https://opendata.dwd.de/climate_environment/CDC/Readme_intro_CDC_ftp.txt</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>All 5 LLs</t>
+          <t>All 5 LLs through raster clipping to LL boundaries</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>vector</t>
+          <t>raster</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Already integrated as committed GeoJSON fixtures and runtime copies.</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>include</t>
-        </is>
-      </c>
+          <t>Bounded CDC entry for spatial precipitation context.</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -4344,7 +4310,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dlr_croptypes</t>
+          <t>buek250_soil</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4354,12 +4320,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DLR Croptypes Germany</t>
+          <t>BUEK250 Soil</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CROPTYPES_DE_P1Y</t>
+          <t>BUEK250 soil polygons</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4374,37 +4340,37 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>annual crop type product</t>
+          <t>static federal soil map</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>OGC-download</t>
+          <t>manual-download</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://geoservice.dlr.de/eoc/ogc/stac/v1/collections/CROPTYPES_DE_P1Y?f=text/html</t>
+          <t>https://www.bgr.bund.de/DE/Themen/Boden/Informationsgrundlagen/Bodenkundliche_Karten_Datenbanken/BUEK250/buek250_node.html</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>COG/STAC</t>
+          <t>GeoPackage/GeoJSON</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>DLR open data terms</t>
+          <t>GeoNutzV/DL-DE-BY style terms</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>annual</t>
+          <t>static</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>https://geoservice.dlr.de/eoc/ogc/stac/v1/collections/CROPTYPES_DE_P1Y?f=text/html</t>
+          <t>https://www.bgr.bund.de/DE/Themen/Boden/Informationsgrundlagen/Bodenkundliche_Karten_Datenbanken/BUEK250/buek250_node.html</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -4414,7 +4380,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>raster</t>
+          <t>vector</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -4424,7 +4390,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Already integrated through the raster PMTiles path.</t>
+          <t>Already integrated as committed GeoJSON fixtures and runtime copies.</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -4439,54 +4405,94 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>inspire_geoportal_iacs</t>
+          <t>dlr_croptypes</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>INSPIRE / Discovery</t>
+          <t>Existing Integrations</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>INSPIRE Geoportal</t>
+          <t>DLR Croptypes Germany</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Targeted IACS/InVeKoS discovery query</t>
+          <t>CROPTYPES_DE_P1Y</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>annual crop type product</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>manual-download</t>
+          <t>OGC-download</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://inspire-geoportal.ec.europa.eu/srv/eng/catalog.search#/home</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
+          <t>https://geoservice.dlr.de/eoc/ogc/stac/v1/collections/CROPTYPES_DE_P1Y?f=text/html</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>COG/STAC</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>DLR open data terms</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>https://inspire-geoportal.ec.europa.eu/srv/eng/catalog.search#/home</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
+          <t>https://geoservice.dlr.de/eoc/ogc/stac/v1/collections/CROPTYPES_DE_P1Y?f=text/html</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>All 5 LLs</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>raster</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Already integrated through the raster PMTiles path.</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -4494,22 +4500,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>europe_land_iacs</t>
+          <t>inspire_geoportal_iacs</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IACS / InVeKoS</t>
+          <t>INSPIRE / Discovery</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Europe-LAND Harmonized IACS Inventory</t>
+          <t>INSPIRE Geoportal</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>European GSA/IACS harmonized inventory</t>
+          <t>Targeted IACS/InVeKoS discovery query</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4517,30 +4523,66 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>EU INSPIRE member-state metadata catalogue</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>metadata records vary by provider</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Zenodo</t>
+          <t>manual-download</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://zenodo.org/records/18670815</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
+          <t>https://inspire-geoportal.ec.europa.eu/srv/eng/catalog.search#/home</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>catalogue metadata; downstream formats vary</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>provider-specific</t>
+        </is>
+      </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>https://zenodo.org/records/18670815</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+          <t>https://inspire-geoportal.ec.europa.eu/srv/eng/catalog.search#/home</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>All 5 LLs as discovery aid only; use state endpoints where possible</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Bounded to targeted IACS/InVeKoS discovery; not an integration source by itself.</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
@@ -4549,7 +4591,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>invekos_brandenburg_dfbk</t>
+          <t>europe_land_iacs</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4559,12 +4601,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>InVeKoS Brandenburg DFBK</t>
+          <t>Europe-LAND Harmonized IACS Inventory</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Digitales Feldblockkataster</t>
+          <t>European GSA/IACS harmonized inventory</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4572,30 +4614,66 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>European Union countries/states represented in record files</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>IACS/GSA years vary by country/state</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>WFS</t>
+          <t>Zenodo</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://isk.geobasis-bb.de/ows/geobroker_l_dfbk_wfs</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
+          <t>https://zenodo.org/records/18670815</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Zenodo files; harmonized IACS inventory</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Zenodo record license</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>record versioned release</t>
+        </is>
+      </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>https://geoportal.brandenburg.de/detailansichtdienst/render?url=https://geoportal.brandenburg.de/gs-json/xml?fileid=9e95f21f-4ecf-4682-9a44-e5f7609f6fa0</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+          <t>https://zenodo.org/records/18670815</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Potentially all 5 LLs; verify German state coverage and file size before download</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Large harmonized inventory; integration must bound downloads to German/LL-relevant files.</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
@@ -4604,7 +4682,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>invekos_hesse_landwirtschaftliche_flaechen</t>
+          <t>invekos_brandenburg_dfbk</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4614,12 +4692,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>InVeKoS Hesse</t>
+          <t>InVeKoS Brandenburg DFBK</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>lawi:LandwirtschaftlicheFlaechen_2024</t>
+          <t>Digitales Feldblockkataster</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4627,8 +4705,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Brandenburg and Berlin</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>annual slices 2010-2026; current service updates continue</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>WFS</t>
@@ -4636,21 +4722,49 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://inspire-geo.ibykus.net/geoserver/lawi/wfs</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+          <t>https://isk.geobasis-bb.de/ows/geobroker_l_dfbk_wfs</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>GML via WFS; ZIP bulk download also available</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>DL-DE-BY-2.0</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>continuous/current plus historical annual slices</t>
+        </is>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>https://inspire-geo.ibykus.net/geoserver/lawi/wfs?service=WFS&amp;version=2.0.0&amp;request=GetCapabilities</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
+          <t>https://geoportal.brandenburg.de/detailansichtdienst/render?url=https://geoportal.brandenburg.de/gs-json/xml?fileid=9e95f21f-4ecf-4682-9a44-e5f7609f6fa0</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>east-brandenburg, havellandisches-luch</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Strong LL fit; use WFS or bulk ZIP and clip after CRS alignment.</t>
+        </is>
+      </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
@@ -4659,7 +4773,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>invekos_hesse_landscape</t>
+          <t>invekos_hesse_landwirtschaftliche_flaechen</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4674,7 +4788,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>lawi:Landschaftselemente_2024</t>
+          <t>lawi:LandwirtschaftlicheFlaechen_2024</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4682,8 +4796,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Hesse</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>WFS</t>
@@ -4694,18 +4816,46 @@
           <t>https://inspire-geo.ibykus.net/geoserver/lawi/wfs</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>GML/SHAPE-ZIP via WFS GetFeature</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>annual layer versions</t>
+        </is>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
           <t>https://inspire-geo.ibykus.net/geoserver/lawi/wfs?service=WFS&amp;version=2.0.0&amp;request=GetCapabilities</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>north-hessian-loess, hessian-low-mountain</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Contractor-hosted WFS; watch dead-URL risk and pin layer year in sources.yaml.</t>
+        </is>
+      </c>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
@@ -4714,7 +4864,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>invekos_hesse_lpis</t>
+          <t>invekos_hesse_landscape</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4729,7 +4879,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>lawi:LPIS-Referenzparzellen_2024</t>
+          <t>lawi:Landschaftselemente_2024</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -4737,8 +4887,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Hesse</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>WFS</t>
@@ -4749,18 +4907,46 @@
           <t>https://inspire-geo.ibykus.net/geoserver/lawi/wfs</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>GML/SHAPE-ZIP via WFS GetFeature</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>annual layer versions</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
           <t>https://inspire-geo.ibykus.net/geoserver/lawi/wfs?service=WFS&amp;version=2.0.0&amp;request=GetCapabilities</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>north-hessian-loess, hessian-low-mountain</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Contractor-hosted WFS; landscape elements are reviewable separately from parcels.</t>
+        </is>
+      </c>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
@@ -4769,7 +4955,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>invekos_niedersachsen_referenzparzellen</t>
+          <t>invekos_hesse_lpis</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4779,12 +4965,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>InVeKoS Niedersachsen</t>
+          <t>InVeKoS Hesse</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Referenzparzellen</t>
+          <t>lawi:LPIS-Referenzparzellen_2024</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -4792,8 +4978,16 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Hesse</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>WFS</t>
@@ -4801,21 +4995,49 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://sla.niedersachsen.de/agrarfoerderung/agrar_ref_inspire/wfs</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+          <t>https://inspire-geo.ibykus.net/geoserver/lawi/wfs</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>GML/SHAPE-ZIP via WFS GetFeature</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>CC BY 4.0</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>annual layer versions</t>
+        </is>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>https://gdi.bmleh.de/geodaten/geodaten-aus-dem-invekos-eu-agrarfoerderung</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
+          <t>https://inspire-geo.ibykus.net/geoserver/lawi/wfs?service=WFS&amp;version=2.0.0&amp;request=GetCapabilities</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>north-hessian-loess, hessian-low-mountain</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Contractor-hosted WFS; LPIS reference parcels are reviewable separately from landscape elements.</t>
+        </is>
+      </c>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
@@ -4824,22 +5046,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>jki_small_structures</t>
+          <t>invekos_niedersachsen_referenzparzellen</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Landscape Structure</t>
+          <t>IACS / InVeKoS</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>JKI Small Structures</t>
+          <t>InVeKoS Niedersachsen</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Small structures database</t>
+          <t>Referenzparzellen</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -4847,30 +5069,66 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Niedersachsen, Bremen, Hamburg</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>manual-download</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://www.julius-kuehn.de/en/small-structures</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+          <t>https://sla.niedersachsen.de/agrarfoerderung/agrar_ref_inspire/wfs</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>GML via WFS GetFeature</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>https://www.julius-kuehn.de/en/small-structures</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
+          <t>https://gdi.bmleh.de/geodaten/geodaten-aus-dem-invekos-eu-agrarfoerderung</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>uelzen</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Endpoint identified through federal overview; license and layer years need confirmation before integration.</t>
+        </is>
+      </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
@@ -4879,22 +5137,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>bfn_protected_areas</t>
+          <t>jki_small_structures</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Protected Areas</t>
+          <t>Landscape Structure</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BfN Schutzgebiete</t>
+          <t>JKI Small Structures</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Federal protected areas WFS</t>
+          <t>Small structures database</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -4902,30 +5160,66 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>WFS</t>
+          <t>manual-download</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://geodienste.bfn.de/ogc/wfs/schutzgebiet</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
+          <t>https://www.julius-kuehn.de/en/small-structures</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>https://gdk.gdi-de.org/geonetwork/srv/api/records/bec888f9-ba0c-42dc-846e-177b8265dafa</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
+          <t>https://www.julius-kuehn.de/en/small-structures</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Potentially all 5 LLs if open geodata access is confirmed</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Approved checkpoint default: keep as needs-verification row; do not backlog until access is confirmed.</t>
+        </is>
+      </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
@@ -4934,22 +5228,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>thuenen_land_use_timeseries</t>
+          <t>bfn_protected_areas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Remote Sensing / Land Use</t>
+          <t>Protected Areas</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Thuenen agricultural land-use time series</t>
+          <t>BfN Schutzgebiete</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Annual agricultural land-use maps 1990-2023</t>
+          <t>Federal protected areas WFS</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -4957,30 +5251,66 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>feature-type specific; current federal protected-area datasets</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Nextcloud</t>
+          <t>WFS</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://cloud.thuenen.de/index.php/s/yLGJNi6MoePycqf</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
+          <t>https://geodienste.bfn.de/ogc/wfs/schutzgebiet</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>GML via WFS GetFeature</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>GeoNutzV</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>annual/product-specific updates</t>
+        </is>
+      </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>https://cloud.thuenen.de/index.php/s/yLGJNi6MoePycqf</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
+          <t>https://gdk.gdi-de.org/geonetwork/srv/api/records/bec888f9-ba0c-42dc-846e-177b8265dafa</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>All 5 LLs</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>vector</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Bounded to protected-area layers relevant for LL context; avoid enumerating full portal breadth.</t>
+        </is>
+      </c>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
@@ -4989,22 +5319,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ugr_ecosystem_atlas</t>
+          <t>thuenen_land_use_timeseries</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>UGR / Ecosystem Accounts</t>
+          <t>Remote Sensing / Land Use</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Destatis UGR Ecosystem Atlas</t>
+          <t>Thuenen agricultural land-use time series</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Ecosystem accounting atlas</t>
+          <t>Annual agricultural land-use maps 1990-2023</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5012,35 +5342,162 @@
           <t>no</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>1990-2023 annual agricultural land-use maps</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>manual-download</t>
+          <t>Zenodo</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://oekosystematlas-ugr.destatis.de/</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
+          <t>https://zenodo.org/records/15055561</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>COG/GeoTIFF record</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Zenodo record license</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>record versioned release</t>
+        </is>
+      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Umwelt/UGR/oekosystemgesamtrechnungen/</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
+          <t>https://zenodo.org/records/15055561</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>All 5 LLs through raster clipping to LL boundaries</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>raster</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Approved checkpoint default: use Zenodo fallback when Nextcloud share is unreachable; temporal comparability still needs review.</t>
+        </is>
+      </c>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ugr_ecosystem_atlas</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>UGR / Ecosystem Accounts</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Destatis UGR Ecosystem Atlas</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ecosystem accounting atlas</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>manual-download</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://oekosystematlas-ugr.destatis.de/</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>static downloads; exact file format needs verification</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>[needs-verification]</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>https://www.destatis.de/DE/Themen/Gesellschaft-Umwelt/Umwelt/UGR/oekosystemgesamtrechnungen/</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>All 5 LLs if municipality or grid data can be joined to LL regions</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>tabular</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>No confirmed API; use Destatis download/publication page and verify exact downloadable format before integration.</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>